<commit_message>
docs(governance): align daily sync and spreadsheet scope
O que é: Atualizar as decisões e o acompanhamento das integrações Majucau.

O que foi feito: BK-027 foi atualizado para 40% após a CI de PostgreSQL e Windows aprovar a allowlist do worker. Backlog e documentos agora dizem que o Bling relê diariamente todas as contas; o checkpoint serve para retomada. XLS e XLSX foram registrados como formatos diários do Drive, ainda pendentes de parser seguro e homologação das abas. Manifesto e planilha oficial foram atualizados.

Próximo passo: Implementar e validar leitura segura em fluxo para Excel; homologar paginação Bling e confirmar o provisionamento das permissões do banco no instalador.

Quanto falta da tarefa BK-027: 60%

Quanto falta da tarefa BK-039: 100%

Quanto falta da tarefa BK-042: 60%

Quanto falta da tarefa BK-043: 60%

Quanto falta do projeto: 88,9%
</commit_message>
<xml_diff>
--- a/artifacts/planejamento/outputs/MAJUCAU_BACKLOG_E_EVOLUCAO_v2.xlsx
+++ b/artifacts/planejamento/outputs/MAJUCAU_BACKLOG_E_EVOLUCAO_v2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evolucao" sheetId="1" r:id="Rec1eff6292a44914"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tarefas" sheetId="2" r:id="R80ee2eb555f94667"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisoes" sheetId="3" r:id="Rb9db71eaf4064902"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura" sheetId="4" r:id="Rfd513f3817c04638"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evolucao" sheetId="1" r:id="Rb6e788992fa64d05"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tarefas" sheetId="2" r:id="R301fad4442c44bc3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisoes" sheetId="3" r:id="R18db7a9e505d4e58"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura" sheetId="4" r:id="Ra5845b94ea594652"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -555,7 +555,7 @@
       </x:c>
       <x:c r="B8" s="23" t="n">
         <x:f>SUM('Tarefas'!$N$6:$N$132)/SUM('Tarefas'!$F$6:$F$132)</x:f>
-        <x:v>0.11031496062992126</x:v>
+        <x:v>0.11070866141732284</x:v>
       </x:c>
       <x:c r="C8" s="11" t="str">
         <x:v>Estimativa; não é prontidão</x:v>
@@ -715,7 +715,7 @@
       </x:c>
       <x:c r="C16" s="26" t="n">
         <x:f>SUMIFS('Tarefas'!$N$6:$N$132,'Tarefas'!$B$6:$B$132,A16)/SUMIFS('Tarefas'!$F$6:$F$132,'Tarefas'!$B$6:$B$132,A16)</x:f>
-        <x:v>0.5</x:v>
+        <x:v>0.5071428571428571</x:v>
       </x:c>
       <x:c r="D16" s="2"/>
       <x:c r="E16" s="2" t="str">
@@ -972,7 +972,7 @@
     </x:row>
     <x:row r="33" ht="28" customHeight="1">
       <x:c r="A33" s="2" t="str">
-        <x:v>Backlog em 13/10/2026: 7 concluídas, 18 em andamento e 102 não iniciadas. Estimativa: 11,0%; restante: 89,0%. É uma estimativa, não prova de prontidão.</x:v>
+        <x:v>Backlog em 13/10/2026: 7 concluídas, 18 em andamento e 102 não iniciadas. Estimativa: 11,1%; restante: 88,9%. É uma estimativa, não prova de prontidão.</x:v>
       </x:c>
       <x:c r="B33" s="2"/>
       <x:c r="C33" s="2"/>
@@ -2405,10 +2405,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G33" s="17" t="n">
-        <x:v>0.35</x:v>
+        <x:v>0.4</x:v>
       </x:c>
       <x:c r="H33" s="12" t="str">
-        <x:v>35%: o worker compõe serviços, limita conexão ao PostgreSQL e encerra de forma controlada; a saúde verifica conexão e quatro tabelas essenciais com códigos sanitizados. A CI 38379095626 aplicou database/privileges/runtime.sql em PostgreSQL descartável e confirmou permissões mínimas do papel runtime, bloqueio de alteração direta de RAW/auditoria e acesso apenas às funções de transição aprovadas. Ainda faltam validar provisionamento das permissões na instalação, configuração de produção e operação em VM limpa. Evidências: docs/evidence/WORKER-DATABASE-SCHEMA-READINESS-2026-10-13.md e docs/evidence/WORKER-RUNTIME-DATABASE-PRIVILEGES-2026-10-13.md.</x:v>
+        <x:v>40%: o worker compõe serviços, limita conexão ao PostgreSQL e encerra de forma controlada; a saúde verifica conexão e quatro tabelas essenciais com códigos sanitizados. A CI 38383732688 passou nos quatro grupos e confirmou em PostgreSQL descartável a lista exata de leitura/escrita, bloqueio de exclusão e de gravação direta em RAW/auditoria, ausência de acessos por coluna ou sequências e execução somente da função de encerramento de versão RAW. Ainda faltam validar o provisionamento dessas permissões na instalação, a configuração de produção e a operação em VM limpa. Evidências: docs/evidence/WORKER-DATABASE-SCHEMA-READINESS-2026-10-13.md e docs/evidence/WORKER-RUNTIME-DATABASE-PRIVILEGES-2026-10-13.md.</x:v>
       </x:c>
       <x:c r="I33" s="11" t="str">
         <x:v>Engenharia</x:v>
@@ -2426,7 +2426,7 @@
       </x:c>
       <x:c r="N33" s="11" t="n">
         <x:f>F33*G33</x:f>
-        <x:v>0.35</x:v>
+        <x:v>0.4</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="72" customHeight="1">
@@ -3066,7 +3066,7 @@
         <x:v>0.4</x:v>
       </x:c>
       <x:c r="H48" s="12" t="str">
-        <x:v>40%: a ponte do Site lista arquivos em páginas e baixa em fluxo, calcula hash, confere a versão e grava staging em blocos. Faltam credencial e pasta reais do Drive, importação controlada, confirmar leitura somente, agenda diária, medição de carga e VM limpa. Evidência: docs/evidence/DRIVE-STREAMING-IMPORT-2026-10-13.md.</x:v>
+        <x:v>40%: a ponte do Site lista arquivos em páginas e baixa em fluxo, calcula hash, confere a versão e grava staging em blocos. Gisele confirmou em 13/10/2026 que os arquivos diários incluem XLS/XLSX, ainda recusados pela ponte. Faltam credencial e pasta reais do Drive, parser de Excel seguro em fluxo, importação controlada, confirmar leitura somente, agenda diária, medição de carga e VM limpa. Evidência: docs/evidence/DRIVE-STREAMING-IMPORT-2026-10-13.md.</x:v>
       </x:c>
       <x:c r="I48" s="10" t="str">
         <x:v>Engenharia</x:v>
@@ -3112,7 +3112,7 @@
         <x:v>0.4</x:v>
       </x:c>
       <x:c r="H49" s="12" t="str">
-        <x:v>40%: estruturas CSV/TSV/JSON são lidas em fluxo com limites e staging; arquivos XLS/XLSX são recusados e nenhuma linha vira fato financeiro antes de aprovação do layout. Faltam contratos aprovados e amostras reais autorizadas, carga e ensaio em VM limpa. Evidência: docs/evidence/DRIVE-STREAMING-IMPORT-2026-10-13.md.</x:v>
+        <x:v>40%: estruturas CSV/TSV/JSON são lidas em fluxo com limites e staging; arquivos XLS/XLSX ainda são recusados. Gisele confirmou em 13/10/2026 que Excel XLS/XLSX faz parte dos arquivos diários do Drive. Nenhuma linha vira fato financeiro antes de aprovação do layout. Faltam parser seguro de Excel, contratos aprovados e amostras reais autorizadas, carga e ensaio em VM limpa. Evidência: docs/evidence/DRIVE-STREAMING-IMPORT-2026-10-13.md.</x:v>
       </x:c>
       <x:c r="I49" s="11" t="str">
         <x:v>Engenharia</x:v>
@@ -6758,7 +6758,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbce0a480ea884dc6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb0ebeac9e4fe4900"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9969,7 +9969,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R73ccbd8125c7463a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbad49d328ecc4c9f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10394,7 +10394,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb94e3244d4a14873"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2f25cbc0e2ee49aa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat(bling): resume API sync from page checkpoints
O que é: Retomada segura da sincronização diária do Bling por página.

O que foi feito: Páginas confirmadas ficam em staging privado; após falha, o retry continua da última página salva. A publicação RAW, a aposentadoria do retrato anterior, o cursor e o sucesso são atômicos. Atualizei permissões, evidências, backlog e quadro de acompanhamento. As telas e regras financeiras aprovadas não mudaram.

Próximo passo: Enviar esta alteração ao GitHub, aguardar a CI e depois homologar a paginação na conta Bling real.

Quanto falta da tarefa: 50%

Quanto falta do projeto: 88,5%
</commit_message>
<xml_diff>
--- a/artifacts/planejamento/outputs/MAJUCAU_BACKLOG_E_EVOLUCAO_v2.xlsx
+++ b/artifacts/planejamento/outputs/MAJUCAU_BACKLOG_E_EVOLUCAO_v2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evolucao" sheetId="1" r:id="Rb6e788992fa64d05"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tarefas" sheetId="2" r:id="R301fad4442c44bc3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisoes" sheetId="3" r:id="R18db7a9e505d4e58"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura" sheetId="4" r:id="Ra5845b94ea594652"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evolucao" sheetId="1" r:id="R7675a02a89df4574"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tarefas" sheetId="2" r:id="Rd8235333ac5443a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisoes" sheetId="3" r:id="R034127754da6401b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura" sheetId="4" r:id="Re85f5bb731f5408d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -475,7 +475,7 @@
     </x:row>
     <x:row r="3" ht="28" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>Status atualizado em 13/10/2026 | fechamento funcional de 13/09/2026</x:v>
+        <x:v>Status atualizado em 18/10/2026 | fechamento funcional de 13/09/2026</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -555,7 +555,7 @@
       </x:c>
       <x:c r="B8" s="23" t="n">
         <x:f>SUM('Tarefas'!$N$6:$N$132)/SUM('Tarefas'!$F$6:$F$132)</x:f>
-        <x:v>0.11070866141732284</x:v>
+        <x:v>0.1152755905511811</x:v>
       </x:c>
       <x:c r="C8" s="11" t="str">
         <x:v>Estimativa; não é prontidão</x:v>
@@ -755,7 +755,7 @@
       </x:c>
       <x:c r="C18" s="26" t="n">
         <x:f>SUMIFS('Tarefas'!$N$6:$N$132,'Tarefas'!$B$6:$B$132,A18)/SUMIFS('Tarefas'!$F$6:$F$132,'Tarefas'!$B$6:$B$132,A18)</x:f>
-        <x:v>0.10333333333333332</x:v>
+        <x:v>0.142</x:v>
       </x:c>
       <x:c r="D18" s="2"/>
       <x:c r="E18" s="2" t="str">
@@ -972,7 +972,7 @@
     </x:row>
     <x:row r="33" ht="28" customHeight="1">
       <x:c r="A33" s="2" t="str">
-        <x:v>Backlog em 13/10/2026: 7 concluídas, 18 em andamento e 102 não iniciadas. Estimativa: 11,1%; restante: 88,9%. É uma estimativa, não prova de prontidão.</x:v>
+        <x:v>Backlog em 18/10/2026: 7 concluídas, 19 em andamento e 101 não iniciadas. Estimativa: 11,5%; restante: 88,5%. É uma estimativa, não prova de prontidão.</x:v>
       </x:c>
       <x:c r="B33" s="2"/>
       <x:c r="C33" s="2"/>
@@ -2923,15 +2923,17 @@
         <x:v>Desenvolvimento</x:v>
       </x:c>
       <x:c r="E45" s="12" t="str">
-        <x:v>Não iniciada</x:v>
+        <x:v>Em andamento</x:v>
       </x:c>
       <x:c r="F45" s="18" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G45" s="17" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H45" s="12" t="str"/>
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="H45" s="12" t="str">
+        <x:v>50%: scheduler diário às 09:30 em America/Sao_Paulo, correlation_id estável, trava PostgreSQL entre instâncias e checkpoints duráveis das páginas Bling. Após interrupção, retoma da próxima página confirmada; publica RAW, encerra páginas antigas e atualiza cursor/sucesso em uma transação final. Falha mantém o retrato anterior e auditoria, com páginas confirmadas disponíveis para retry. Testes do pacote passaram em PostgreSQL 18 descartável com permissões runtime verificadas. Ainda faltam provar o fim da paginação na conta real, integrar o Drive, operar continuamente e homologar. docs/evidence/BLING-PAGE-CHECKPOINTS-2026-10-18.md</x:v>
+      </x:c>
       <x:c r="I45" s="11" t="str">
         <x:v>Engenharia</x:v>
       </x:c>
@@ -2950,7 +2952,7 @@
       </x:c>
       <x:c r="N45" s="11" t="n">
         <x:f>F45*G45</x:f>
-        <x:v>0</x:v>
+        <x:v>0.5</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="72" customHeight="1">
@@ -3017,10 +3019,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G47" s="17" t="n">
-        <x:v>0.75</x:v>
+        <x:v>0.78</x:v>
       </x:c>
       <x:c r="H47" s="12" t="str">
-        <x:v>75%: leitura de receber, pagar e movimentações de caixa com GET limitado; OAuth local via callback HTTPS, state e DPAPI. /caixas usa parâmetros documentados e limite local. Faltam integração/persistência de caixa, homologação da conta, término da paginação e cursor incremental. Evidência: docs/evidence/BLING-OAUTH-LOCAL-RELAY-2026-10-13.md.</x:v>
+        <x:v>78%: leitura de receber, pagar e movimentações de caixa com GET limitado; OAuth local via callback HTTPS, state e DPAPI. /caixas usa parâmetros documentados e limite local. Sem metadados, continua após páginas curtas e trata data: [] como marcador provisório de término. Falta confirmar esse comportamento na conta real, integrar/persistir caixa, homologar categorias/campos, retomar cursor incremental e concluir sincronização real. Evidência: docs/evidence/BLING-PAGINATION-CONTRACT-2026-10-11.md.</x:v>
       </x:c>
       <x:c r="I47" s="11" t="str">
         <x:v>Engenharia</x:v>
@@ -3040,7 +3042,7 @@
       </x:c>
       <x:c r="N47" s="11" t="n">
         <x:f>F47*G47</x:f>
-        <x:v>0.75</x:v>
+        <x:v>0.78</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="72" customHeight="1">
@@ -3063,10 +3065,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G48" s="16" t="n">
-        <x:v>0.4</x:v>
+        <x:v>0.45</x:v>
       </x:c>
       <x:c r="H48" s="12" t="str">
-        <x:v>40%: a ponte do Site lista arquivos em páginas e baixa em fluxo, calcula hash, confere a versão e grava staging em blocos. Gisele confirmou em 13/10/2026 que os arquivos diários incluem XLS/XLSX, ainda recusados pela ponte. Faltam credencial e pasta reais do Drive, parser de Excel seguro em fluxo, importação controlada, confirmar leitura somente, agenda diária, medição de carga e VM limpa. Evidência: docs/evidence/DRIVE-STREAMING-IMPORT-2026-10-13.md.</x:v>
+        <x:v>45% (estimativa): o núcleo Go de listagem e download GET em fluxo, restrito por IDs das três pastas, e o provedor de token de service account via cofre foram implementados e testados localmente. Ainda faltam credenciais/IDs reais, integração ao worker/jobs/armazenamento, contratos e importação real; XLS/XLSX continuam sem parser seguro. Evidência: docs/evidence/GOOGLE-DRIVE-READ-ADAPTER-2026-10-18.md.</x:v>
       </x:c>
       <x:c r="I48" s="10" t="str">
         <x:v>Engenharia</x:v>
@@ -3086,7 +3088,7 @@
       </x:c>
       <x:c r="N48" s="10" t="n">
         <x:f>F48*G48</x:f>
-        <x:v>0.4</x:v>
+        <x:v>0.45</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="72" customHeight="1">
@@ -6758,7 +6760,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb0ebeac9e4fe4900"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd859c0794a7042cd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9969,7 +9971,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbad49d328ecc4c9f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra1fcf46f4a544409"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10394,7 +10396,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2f25cbc0e2ee49aa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d57b14109844a6d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat(googledrive): stage verified files privately
O que é: etapa privada e temporária para processar arquivos do Drive em fluxo.

O que foi feito: criado WithPrivateStage para baixar arquivos verificados em diretório privado, entregar o conteúdo como fluxo ao processador, limpar o temporário e reiniciar bytes incompletos em retry. Atualizados o backlog, a planilha oficial, o registro da etapa e a governança. Telas e regras financeiras não foram alteradas.

Próximo passo: ligar o estágio aos importadores após homologar contratos e amostras; configurar Drive e criar suporte seguro a XLS/XLSX.

Quanto falta da tarefa BK-042: 42%.

Quanto falta do projeto: 88,4%.
</commit_message>
<xml_diff>
--- a/artifacts/planejamento/outputs/MAJUCAU_BACKLOG_E_EVOLUCAO_v2.xlsx
+++ b/artifacts/planejamento/outputs/MAJUCAU_BACKLOG_E_EVOLUCAO_v2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evolucao" sheetId="1" r:id="R7675a02a89df4574"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tarefas" sheetId="2" r:id="Rd8235333ac5443a8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisoes" sheetId="3" r:id="R034127754da6401b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura" sheetId="4" r:id="Re85f5bb731f5408d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evolucao" sheetId="1" r:id="Rf97ebd6f8a324367"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tarefas" sheetId="2" r:id="R6f90e6ce0166417f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisoes" sheetId="3" r:id="Rdb26a564b9ee4e2e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura" sheetId="4" r:id="Rf073d2e3ec48413f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -555,7 +555,7 @@
       </x:c>
       <x:c r="B8" s="23" t="n">
         <x:f>SUM('Tarefas'!$N$6:$N$132)/SUM('Tarefas'!$F$6:$F$132)</x:f>
-        <x:v>0.1152755905511811</x:v>
+        <x:v>0.1162992125984252</x:v>
       </x:c>
       <x:c r="C8" s="11" t="str">
         <x:v>Estimativa; não é prontidão</x:v>
@@ -755,7 +755,7 @@
       </x:c>
       <x:c r="C18" s="26" t="n">
         <x:f>SUMIFS('Tarefas'!$N$6:$N$132,'Tarefas'!$B$6:$B$132,A18)/SUMIFS('Tarefas'!$F$6:$F$132,'Tarefas'!$B$6:$B$132,A18)</x:f>
-        <x:v>0.142</x:v>
+        <x:v>0.15066666666666664</x:v>
       </x:c>
       <x:c r="D18" s="2"/>
       <x:c r="E18" s="2" t="str">
@@ -972,7 +972,7 @@
     </x:row>
     <x:row r="33" ht="28" customHeight="1">
       <x:c r="A33" s="2" t="str">
-        <x:v>Backlog em 18/10/2026: 7 concluídas, 19 em andamento e 101 não iniciadas. Estimativa: 11,5%; restante: 88,5%. É uma estimativa, não prova de prontidão.</x:v>
+        <x:v>Backlog em 18/10/2026: 7 concluídas, 19 em andamento e 101 não iniciadas. Estimativa: 11,6%; restante: 88,4%. É uma estimativa, não prova de prontidão.</x:v>
       </x:c>
       <x:c r="B33" s="2"/>
       <x:c r="C33" s="2"/>
@@ -3065,10 +3065,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G48" s="16" t="n">
-        <x:v>0.45</x:v>
+        <x:v>0.58</x:v>
       </x:c>
       <x:c r="H48" s="12" t="str">
-        <x:v>45% (estimativa): o núcleo Go de listagem e download GET em fluxo, restrito por IDs das três pastas, e o provedor de token de service account via cofre foram implementados e testados localmente. Ainda faltam credenciais/IDs reais, integração ao worker/jobs/armazenamento, contratos e importação real; XLS/XLSX continuam sem parser seguro. Evidência: docs/evidence/GOOGLE-DRIVE-READ-ADAPTER-2026-10-18.md.</x:v>
+        <x:v>58% (estimativa): o núcleo GET do Drive lista e baixa em fluxo, mantém checkpoints/páginas e versões de metadados e publica o inventário de forma atômica. O worker agenda a listagem diária das três pastas às 09:30 quando IDs e credencial DPAPI estão configurados, com correlação estável por dia/pasta e falha independente por origem. Nesta atualização, `WithPrivateStage` grava o download verificado numa pasta temporária privada, expõe o conteúdo como `io.Reader` ao callback e limpa o temporário ao terminar; retry substitui bytes incompletos e erros de limpeza preservam caminho tipado sem expô-lo na mensagem comum. `go test ./... -count=1`, `go vet ./...`, `go mod verify`, verificação do backlog, limites Go e `git diff --check` passaram no Windows. O novo estágio ainda não foi ligado ao worker ou a importadores homologados. Ainda faltam contratos e amostras, credenciais/IDs reais, importação e homologação; XLS/XLSX continuam sem parser seguro. Evidências: docs/evidence/GOOGLE-DRIVE-READ-ADAPTER-2026-10-18.md, docs/evidence/GOOGLE-DRIVE-DAILY-WORKER-2026-10-18.md e docs/evidence/GOOGLE-DRIVE-PRIVATE-STAGING-2026-10-18.md.</x:v>
       </x:c>
       <x:c r="I48" s="10" t="str">
         <x:v>Engenharia</x:v>
@@ -3088,7 +3088,7 @@
       </x:c>
       <x:c r="N48" s="10" t="n">
         <x:f>F48*G48</x:f>
-        <x:v>0.45</x:v>
+        <x:v>0.58</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="72" customHeight="1">
@@ -6760,7 +6760,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd859c0794a7042cd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R345509b9ad774a24"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9971,7 +9971,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra1fcf46f4a544409"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb6207d6452824cb2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10396,7 +10396,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d57b14109844a6d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc048d23c5e1b4768"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
fix(bling): show missing app secret accurately
O que é: corrigir o estado visual enganoso do Client Secret do Bling.

O que foi feito: a tela passou a usar a confirmação real do cofre, pedir o segredo quando ausente e esclarecer que ele não é a senha do site. Testes e registros de governança foram atualizados; layout e regras financeiras foram preservados.

Próximo passo: cadastrar o Client Secret do aplicativo no Majucau, salvar, autorizar e testar antes de sincronizar dados reais.

Quanto falta da tarefa BK-041: 22%.

Quanto falta do projeto: 88,4%.
</commit_message>
<xml_diff>
--- a/artifacts/planejamento/outputs/MAJUCAU_BACKLOG_E_EVOLUCAO_v2.xlsx
+++ b/artifacts/planejamento/outputs/MAJUCAU_BACKLOG_E_EVOLUCAO_v2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evolucao" sheetId="1" r:id="Rf97ebd6f8a324367"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tarefas" sheetId="2" r:id="R6f90e6ce0166417f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisoes" sheetId="3" r:id="Rdb26a564b9ee4e2e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura" sheetId="4" r:id="Rf073d2e3ec48413f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evolucao" sheetId="1" r:id="R02b4fa02adfe41e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tarefas" sheetId="2" r:id="R8a731aa248bd4c37"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisoes" sheetId="3" r:id="R31773e5ad0d84e9c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura" sheetId="4" r:id="R9ec27f0097c34034"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3022,7 +3022,7 @@
         <x:v>0.78</x:v>
       </x:c>
       <x:c r="H47" s="12" t="str">
-        <x:v>78%: leitura de receber, pagar e movimentações de caixa com GET limitado; OAuth local via callback HTTPS, state e DPAPI. /caixas usa parâmetros documentados e limite local. Sem metadados, continua após páginas curtas e trata data: [] como marcador provisório de término. Falta confirmar esse comportamento na conta real, integrar/persistir caixa, homologar categorias/campos, retomar cursor incremental e concluir sincronização real. Evidência: docs/evidence/BLING-PAGINATION-CONTRACT-2026-10-11.md.</x:v>
+        <x:v>78%: GET/OAuth/DPAPI implementados. Fim desconhecido falha com segurança e preserva snapshot/cursor. Ainda faltam Client Secret real, autorização e integração dos dados aos relatórios.</x:v>
       </x:c>
       <x:c r="I47" s="11" t="str">
         <x:v>Engenharia</x:v>
@@ -6760,7 +6760,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R345509b9ad774a24"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b9d315d86bc4a31"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9971,7 +9971,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb6207d6452824cb2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re65b4a6a55884d9b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10396,7 +10396,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc048d23c5e1b4768"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R21ca33cf65bd40d8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat(import): add isolated streaming xlsx reader
O que é: avanço parcial da BK-043 para leitura segura de arquivos XLSX.

O que foi feito: criado leitor de planilhas XLSX que entrega linhas em fluxo, aplica limites de tamanho, conteúdo descompactado, abas, linhas, colunas e células, rejeita macros e relações externas, não calcula fórmulas e usa índice temporário privado. Corrigida a associação dos caminhos das abas e adicionadas evidências, testes sintéticos e atualização do acompanhamento.

Próximo passo: integrar ao importador do Drive, suportar XLS legado e homologar contratos/amostras autorizadas antes de publicar dados financeiros.

Quanto falta da tarefa BK-043: 60%.

Quanto falta do projeto: 88,4%.
</commit_message>
<xml_diff>
--- a/artifacts/planejamento/outputs/MAJUCAU_BACKLOG_E_EVOLUCAO_v2.xlsx
+++ b/artifacts/planejamento/outputs/MAJUCAU_BACKLOG_E_EVOLUCAO_v2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evolucao" sheetId="1" r:id="R02b4fa02adfe41e1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tarefas" sheetId="2" r:id="R8a731aa248bd4c37"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisoes" sheetId="3" r:id="R31773e5ad0d84e9c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura" sheetId="4" r:id="R9ec27f0097c34034"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evolucao" sheetId="1" r:id="R5186a35fc80e4034"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tarefas" sheetId="2" r:id="R0ab2067e0dc34dc9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisoes" sheetId="3" r:id="Rbcb05fee8c1842b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura" sheetId="4" r:id="R7f133100b6f14059"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3114,7 +3114,7 @@
         <x:v>0.4</x:v>
       </x:c>
       <x:c r="H49" s="12" t="str">
-        <x:v>40%: estruturas CSV/TSV/JSON são lidas em fluxo com limites e staging; arquivos XLS/XLSX ainda são recusados. Gisele confirmou em 13/10/2026 que Excel XLS/XLSX faz parte dos arquivos diários do Drive. Nenhuma linha vira fato financeiro antes de aprovação do layout. Faltam parser seguro de Excel, contratos aprovados e amostras reais autorizadas, carga e ensaio em VM limpa. Evidência: docs/evidence/DRIVE-STREAMING-IMPORT-2026-10-13.md.</x:v>
+        <x:v>40% mantido. Leitor XLSX isolado, testado com dados sintéticos, ainda não integrado ao Drive; XLS não suportado. Faltam integração, contrato das planilhas e homologação real. Nenhuma regra financeira foi alterada. Evidências: docs/evidence/DRIVE-STREAMING-IMPORT-2026-10-13.md e docs/evidence/EXCEL-STREAMING-PARSER-PROTOTYPE-2026-10-18.md.</x:v>
       </x:c>
       <x:c r="I49" s="11" t="str">
         <x:v>Engenharia</x:v>
@@ -6760,7 +6760,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b9d315d86bc4a31"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R728773bd97d046e5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9971,7 +9971,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re65b4a6a55884d9b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfee8dbd42da44004"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10396,7 +10396,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R21ca33cf65bd40d8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref3c1b566b0f4830"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat(financial): add guarded DRE arithmetic
O que é: base do cálculo da DRE própria nas linhas já aprovadas.

O que foi feito: implementei cálculo exato para valores previamente classificados, período e versão obrigatórios, propagação de dados indisponíveis e falha atômica em overflow. Acrescentei casos de referência e atualizei governança, evidência, backlog e planilha.

Próximo passo: ligar os lançamentos reais já classificados, validar o mapeamento do plano de contas com a contabilidade e conciliar por competência.

Quanto falta da tarefa: 95%

Quanto falta do projeto: 88,2%
</commit_message>
<xml_diff>
--- a/artifacts/planejamento/outputs/MAJUCAU_BACKLOG_E_EVOLUCAO_v2.xlsx
+++ b/artifacts/planejamento/outputs/MAJUCAU_BACKLOG_E_EVOLUCAO_v2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evolucao" sheetId="1" r:id="R4e7e4e18b76c4ee3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tarefas" sheetId="2" r:id="Rc01e3565afb845b6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisoes" sheetId="3" r:id="R502c8795a2054eda"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura" sheetId="4" r:id="R8981f215f78f45ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evolucao" sheetId="1" r:id="R9bbe1006b38a4a7c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tarefas" sheetId="2" r:id="R253ca5e88bcd4a0f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisoes" sheetId="3" r:id="R2b1c22e027334c69"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura" sheetId="4" r:id="R859b683865c44bec"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -475,7 +475,7 @@
     </x:row>
     <x:row r="3" ht="28" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>Status atualizado em 18/10/2026 | fechamento funcional de 13/09/2026</x:v>
+        <x:v>Status atualizado em 19/10/2026 | fechamento funcional de 13/09/2026</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -555,7 +555,7 @@
       </x:c>
       <x:c r="B8" s="23" t="n">
         <x:f>SUM('Tarefas'!$N$6:$N$132)/SUM('Tarefas'!$F$6:$F$132)</x:f>
-        <x:v>0.11724409448818898</x:v>
+        <x:v>0.11779527559055118</x:v>
       </x:c>
       <x:c r="C8" s="11" t="str">
         <x:v>Estimativa; não é prontidão</x:v>
@@ -755,7 +755,7 @@
       </x:c>
       <x:c r="C18" s="26" t="n">
         <x:f>SUMIFS('Tarefas'!$N$6:$N$132,'Tarefas'!$B$6:$B$132,A18)/SUMIFS('Tarefas'!$F$6:$F$132,'Tarefas'!$B$6:$B$132,A18)</x:f>
-        <x:v>0.15866666666666665</x:v>
+        <x:v>0.16</x:v>
       </x:c>
       <x:c r="D18" s="2"/>
       <x:c r="E18" s="2" t="str">
@@ -793,7 +793,7 @@
       </x:c>
       <x:c r="C20" s="26" t="n">
         <x:f>SUMIFS('Tarefas'!$N$6:$N$132,'Tarefas'!$B$6:$B$132,A20)/SUMIFS('Tarefas'!$F$6:$F$132,'Tarefas'!$B$6:$B$132,A20)</x:f>
-        <x:v>0.017857142857142856</x:v>
+        <x:v>0.02142857142857143</x:v>
       </x:c>
       <x:c r="D20" s="2"/>
       <x:c r="E20" s="2" t="str">
@@ -972,7 +972,7 @@
     </x:row>
     <x:row r="33" ht="28" customHeight="1">
       <x:c r="A33" s="2" t="str">
-        <x:v>Backlog em 18/10/2026: 7 concluídas, 19 em andamento e 101 não iniciadas. Estimativa: 11,7%; restante: 88,3%. É uma estimativa, não prova de prontidão.</x:v>
+        <x:v>Backlog em 19/10/2026: 7 concluídas, 20 em andamento e 100 não iniciadas. Estimativa: 11,8%; restante: 88,2%. É uma estimativa, não prova de prontidão.</x:v>
       </x:c>
       <x:c r="B33" s="2"/>
       <x:c r="C33" s="2"/>
@@ -3065,10 +3065,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G48" s="16" t="n">
-        <x:v>0.68</x:v>
+        <x:v>0.7</x:v>
       </x:c>
       <x:c r="H48" s="12" t="str">
-        <x:v>68% (estimativa): o worker lê as três raízes às 09:30, percorre subpastas internas com estado por pasta e página, retoma após falha e só publica o inventário completo. O download é protegido por staging privado, conferência de tamanho/checksum/versão e origem; o caminho CSV de recebimentos futuros está ligado à importação parcial idempotente, com arquivos antigos e fontes incompatíveis marcados como pendentes. A prévia autorizada mostrou a raiz real `Meu Drive/MAJUCAU_INTELLIGENCE_INPUT` e a subpasta `03_nuvem_envio/Frete`; os IDs ficam fora do Git. `go test . ./cmd/... ./database/... ./internal/...`, `go vet`, `go mod verify`, verificações de backlog, migrations, limites Go e `git diff --check` passaram localmente. O teste PostgreSQL de árvore aninhada/retomada foi incluído na CI, ainda aguardando execução. Nenhum arquivo real foi baixado ou valor financeiro importado; o CSV disponível estava desatualizado. Faltam provisionar identidade técnica e credencial DPAPI, configurar os IDs localmente, validar a primeira sincronização real, homologar contratos e formatos; XLS/XLSX, TSV/JSON e medição em VM permanecem pendentes. Evidência: docs/evidence/GOOGLE-DRIVE-NESTED-IMPORT-2026-10-18.md.</x:v>
+        <x:v>70% (estimativa): o worker lê as três raízes às 09:30, percorre subpastas com estado por pasta e página, retoma após falha e só publica o inventário completo. O download usa staging privado e confere tamanho, checksum, versão e origem. CSV de recebimentos futuros pode ser importado com atomicidade e idempotência. XLSX agora é baixado em staging privado, limitado a 256 MiB, verificado estruturalmente por streaming, com linhas descartadas sem interpretar fórmulas e temporários removidos; mesmo válido fica pendente até existir contrato financeiro aprovado. Arquivos de outras estruturas e formatos ainda não homologados permanecem pendentes. A conta humana de referência confirmada é financeiro@majucau.com.br e a pasta aprovada foi localizada. A listagem de 18/10/2026 mostrou um XLSX em perdas operacionais e CSVs nas pastas de recebimentos futuros e frete, todos modificados em 11/09/2026; nenhum conteúdo foi baixado ou importado. A identidade técnica de serviço, credencial DPAPI e configuração dos IDs reais ainda faltam para executar a sincronização pelo Majucau. A verificação completa scripts/verify.ps1 passou localmente: suíte Go, go vet, sqlc, migrations, scan de secrets, checks do instalador, lint, typecheck, 33 testes de interface, build e npm audit sem vulnerabilidades. govulncheck não encontrou chamadas vulneráveis; mantém um aviso de módulo para openpgp não usado, sem correção disponível, já registrado em docs/evidence/DEPENDENCY-SECURITY-REMEDIATION-2026-10-10.md. A CI #674 falhou porque faltava versionar o modelo sqlc da migration 000009; o modelo foi regenerado e versionado. A CI #675 passou nos quatro jobs: backlog, mudanças, PostgreSQL e Windows (https://github.com/guilhermejacyzin/majucau/actions/runs/39193226200). Evidência: docs/evidence/GOOGLE-DRIVE-NESTED-IMPORT-2026-10-18.md. Em 19/10/2026, o caminho de provisionamento local foi implementado: chave e IDs em arquivo separado, validação, cofre DPAPI atômico, Named Pipe autenticado por SID e auditoria PostgreSQL sanitizada; erros de auditoria tentam restaurar a configuração anterior. Suítes focadas e scripts/verify.ps1 passaram localmente; TSV da pasta de recebimentos futuros agora passa por validação estrutural em fluxo, com limite de 1 MiB/campo, 4 MiB/registro e 256 campos, sem gerar fatos financeiros. O BK-042 permanece em 70% até provisionar identidade/IDs reais, executar leitura real completa e homologar os contratos de arquivo restantes. A CI #680 passou nos quatro jobs do GitHub Actions em 19/10/2026, incluindo testes Windows, migration/permissões PostgreSQL, backlog e build do pacote.</x:v>
       </x:c>
       <x:c r="I48" s="10" t="str">
         <x:v>Engenharia</x:v>
@@ -3088,7 +3088,7 @@
       </x:c>
       <x:c r="N48" s="10" t="n">
         <x:f>F48*G48</x:f>
-        <x:v>0.68</x:v>
+        <x:v>0.7</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="72" customHeight="1">
@@ -3114,7 +3114,7 @@
         <x:v>0.4</x:v>
       </x:c>
       <x:c r="H49" s="12" t="str">
-        <x:v>40% mantido. Leitor XLSX isolado, testado com dados sintéticos, ainda não integrado ao Drive; XLS não suportado. Faltam integração, contrato das planilhas e homologação real. Nenhuma regra financeira foi alterada. Evidências: docs/evidence/DRIVE-STREAMING-IMPORT-2026-10-13.md e docs/evidence/EXCEL-STREAMING-PARSER-PROTOTYPE-2026-10-18.md.</x:v>
+        <x:v>40% mantido. O XLSX está integrado ao staging do Drive em 02_nuvem_pago/recebimentos_futuros e passa por validação estrutural em streaming, sem interpretar fórmulas ou publicar fatos; permanece pendente até homologar o contrato. O TSV também passa por validação estrutural linha a linha com limites explícitos e permanece pendente até aprovação do contrato. CSV é importado somente na estrutura de recebimentos futuros com o contrato já aprovado. XLS ainda não tem parser; JSON e arquivos das outras estruturas continuam sem interpretação financeira. Faltam identidade técnica, contratos restantes e homologação real; nenhuma regra financeira foi alterada. Evidências: docs/evidence/DRIVE-STREAMING-IMPORT-2026-10-13.md, docs/evidence/EXCEL-STREAMING-PARSER-PROTOTYPE-2026-10-18.md e docs/evidence/DRIVE-TSV-STREAMING-PENDING-2026-10-19.md.</x:v>
       </x:c>
       <x:c r="I49" s="11" t="str">
         <x:v>Engenharia</x:v>
@@ -4107,15 +4107,17 @@
         <x:v>Desenvolvimento</x:v>
       </x:c>
       <x:c r="E72" s="12" t="str">
-        <x:v>Não iniciada</x:v>
+        <x:v>Em andamento</x:v>
       </x:c>
       <x:c r="F72" s="18" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G72" s="16" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H72" s="12" t="str"/>
+        <x:v>0.05</x:v>
+      </x:c>
+      <x:c r="H72" s="12" t="str">
+        <x:v>5%: cálculo puro das linhas aprovadas implementado em internal/financial/dre.go com valores previamente classificados, período explícito, moeda decimal exata e propagação de indisponibilidade; casos de referência, ausência e overflow em dre_test.go. Sem leitura real, mapeamento de contas, publicação de snapshot ou confirmação contábil.</x:v>
+      </x:c>
       <x:c r="I72" s="10" t="str">
         <x:v>Engenharia</x:v>
       </x:c>
@@ -4134,7 +4136,7 @@
       </x:c>
       <x:c r="N72" s="10" t="n">
         <x:f>F72*G72</x:f>
-        <x:v>0</x:v>
+        <x:v>0.05</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="72" customHeight="1">
@@ -6760,7 +6762,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R316e538d9a514157"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd9b439e3625447ec"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9971,7 +9973,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfedaaa5b7ddf4e24"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b5ad6b2dc6c4cfb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10396,7 +10398,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8cd6d07ff1f24fcf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc90b8197d3cf4b9b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat(drive): validar estruturalmente ocorrências e frete em fluxo
O que é: etapa de segurança para examinar arquivos das pastas de perdas operacionais e frete do Drive.
O que foi feito: validei CSV, TSV, JSON, XLS e XLSX em fluxo, um arquivo por vez em área temporária privada; apliquei limites de segurança aos CSVs com vírgula e ponto e vírgula; deixei os valores financeiros sem interpretação; gravei somente contagens e situação no PostgreSQL com repetição idempotente; atualizei a planilha e o registro do backlog. Nenhuma tela ou regra financeira mudou e nenhum arquivo real foi importado.
Próximo passo: confirmar a gravação e repetição do estado no teste PostgreSQL da CI; depois provisionar a identidade técnica do Drive e homologar os contratos antes da importação real.
Quanto falta da tarefa BK-042: 30%.
Quanto falta da tarefa BK-043: 60%.
Quanto falta do projeto: 88,2%.
</commit_message>
<xml_diff>
--- a/artifacts/planejamento/outputs/MAJUCAU_BACKLOG_E_EVOLUCAO_v2.xlsx
+++ b/artifacts/planejamento/outputs/MAJUCAU_BACKLOG_E_EVOLUCAO_v2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evolucao" sheetId="1" r:id="R9bbe1006b38a4a7c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tarefas" sheetId="2" r:id="R253ca5e88bcd4a0f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisoes" sheetId="3" r:id="R2b1c22e027334c69"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura" sheetId="4" r:id="R859b683865c44bec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evolucao" sheetId="1" r:id="R7de97e5ae62c4b87"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tarefas" sheetId="2" r:id="R6b31957099564b38"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisoes" sheetId="3" r:id="R2c6fb1c228ba42d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura" sheetId="4" r:id="R76a2cb10dda240e4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3068,7 +3068,7 @@
         <x:v>0.7</x:v>
       </x:c>
       <x:c r="H48" s="12" t="str">
-        <x:v>70% (estimativa): o worker lê as três raízes às 09:30, percorre subpastas com estado por pasta e página, retoma após falha e só publica o inventário completo. O download usa staging privado e confere tamanho, checksum, versão e origem. CSV de recebimentos futuros pode ser importado com atomicidade e idempotência. XLSX agora é baixado em staging privado, limitado a 256 MiB, verificado estruturalmente por streaming, com linhas descartadas sem interpretar fórmulas e temporários removidos; mesmo válido fica pendente até existir contrato financeiro aprovado. Arquivos de outras estruturas e formatos ainda não homologados permanecem pendentes. A conta humana de referência confirmada é financeiro@majucau.com.br e a pasta aprovada foi localizada. A listagem de 18/10/2026 mostrou um XLSX em perdas operacionais e CSVs nas pastas de recebimentos futuros e frete, todos modificados em 11/09/2026; nenhum conteúdo foi baixado ou importado. A identidade técnica de serviço, credencial DPAPI e configuração dos IDs reais ainda faltam para executar a sincronização pelo Majucau. A verificação completa scripts/verify.ps1 passou localmente: suíte Go, go vet, sqlc, migrations, scan de secrets, checks do instalador, lint, typecheck, 33 testes de interface, build e npm audit sem vulnerabilidades. govulncheck não encontrou chamadas vulneráveis; mantém um aviso de módulo para openpgp não usado, sem correção disponível, já registrado em docs/evidence/DEPENDENCY-SECURITY-REMEDIATION-2026-10-10.md. A CI #674 falhou porque faltava versionar o modelo sqlc da migration 000009; o modelo foi regenerado e versionado. A CI #675 passou nos quatro jobs: backlog, mudanças, PostgreSQL e Windows (https://github.com/guilhermejacyzin/majucau/actions/runs/39193226200). Evidência: docs/evidence/GOOGLE-DRIVE-NESTED-IMPORT-2026-10-18.md. Em 19/10/2026, o caminho de provisionamento local foi implementado: chave e IDs em arquivo separado, validação, cofre DPAPI atômico, Named Pipe autenticado por SID e auditoria PostgreSQL sanitizada; erros de auditoria tentam restaurar a configuração anterior. Suítes focadas e scripts/verify.ps1 passaram localmente; TSV da pasta de recebimentos futuros agora passa por validação estrutural em fluxo, com limite de 1 MiB/campo, 4 MiB/registro e 256 campos, sem gerar fatos financeiros. O BK-042 permanece em 70% até provisionar identidade/IDs reais, executar leitura real completa e homologar os contratos de arquivo restantes. A CI #680 passou nos quatro jobs do GitHub Actions em 19/10/2026, incluindo testes Windows, migration/permissões PostgreSQL, backlog e build do pacote.</x:v>
+        <x:v>70% (estimativa): o worker lê as três raízes às 09:30, percorre subpastas com estado por pasta e página, retoma após falha e só publica o inventário completo. O download usa staging privado e confere tamanho, checksum, versão e origem. CSV de recebimentos futuros pode ser importado com atomicidade e idempotência. XLSX agora é baixado em staging privado, limitado a 256 MiB, verificado estruturalmente por streaming, com linhas descartadas sem interpretar fórmulas e temporários removidos; mesmo válido fica pendente até existir contrato financeiro aprovado. Arquivos de outras estruturas e formatos ainda não homologados permanecem pendentes. A conta humana de referência confirmada é financeiro@majucau.com.br e a pasta aprovada foi localizada. A listagem de 18/10/2026 mostrou um XLSX em perdas operacionais e CSVs nas pastas de recebimentos futuros e frete, todos modificados em 11/09/2026; nenhum conteúdo foi baixado ou importado. A identidade técnica de serviço, credencial DPAPI e configuração dos IDs reais ainda faltam para executar a sincronização pelo Majucau. A verificação completa scripts/verify.ps1 passou localmente: suíte Go, go vet, sqlc, migrations, scan de secrets, checks do instalador, lint, typecheck, 33 testes de interface, build e npm audit sem vulnerabilidades. govulncheck não encontrou chamadas vulneráveis; mantém um aviso de módulo para openpgp não usado, sem correção disponível, já registrado em docs/evidence/DEPENDENCY-SECURITY-REMEDIATION-2026-10-10.md. A CI #674 falhou porque faltava versionar o modelo sqlc da migration 000009; o modelo foi regenerado e versionado. A CI #675 passou nos quatro jobs: backlog, mudanças, PostgreSQL e Windows (https://github.com/guilhermejacyzin/majucau/actions/runs/39193226200). Evidência: docs/evidence/GOOGLE-DRIVE-NESTED-IMPORT-2026-10-18.md. Em 19/10/2026, o caminho de provisionamento local foi implementado: chave e IDs em arquivo separado, validação, cofre DPAPI atômico, Named Pipe autenticado por SID e auditoria PostgreSQL sanitizada; erros de auditoria tentam restaurar a configuração anterior. Suítes focadas e scripts/verify.ps1 passaram localmente; TSV da pasta de recebimentos futuros agora passa por validação estrutural em fluxo, com limite de 1 MiB/campo, 4 MiB/registro e 256 campos, sem gerar fatos financeiros. O BK-042 permanece em 70% até provisionar identidade/IDs reais, executar leitura real completa e homologar os contratos de arquivo restantes. A CI #680 passou nos quatro jobs do GitHub Actions em 19/10/2026, incluindo testes Windows, migration/permissões PostgreSQL, backlog e build do pacote. Em 19/10, a validação estrutural em fluxo das três pastas aprovadas foi ampliada: perdas e frete agora também passam por CSV/TSV/JSON/XLS/XLSX, e o PostgreSQL guarda apenas contagens e estado idempotentes. Nenhum arquivo real foi processado; o teste PostgreSQL desta tabela foi adicionado e aguarda CI porque não há DSN local.</x:v>
       </x:c>
       <x:c r="I48" s="10" t="str">
         <x:v>Engenharia</x:v>
@@ -3114,7 +3114,7 @@
         <x:v>0.4</x:v>
       </x:c>
       <x:c r="H49" s="12" t="str">
-        <x:v>40% mantido. O XLSX está integrado ao staging do Drive em 02_nuvem_pago/recebimentos_futuros e passa por validação estrutural em streaming, sem interpretar fórmulas ou publicar fatos; permanece pendente até homologar o contrato. O TSV também passa por validação estrutural linha a linha com limites explícitos e permanece pendente até aprovação do contrato. CSV é importado somente na estrutura de recebimentos futuros com o contrato já aprovado. XLS ainda não tem parser; JSON e arquivos das outras estruturas continuam sem interpretação financeira. Faltam identidade técnica, contratos restantes e homologação real; nenhuma regra financeira foi alterada. Evidências: docs/evidence/DRIVE-STREAMING-IMPORT-2026-10-13.md, docs/evidence/EXCEL-STREAMING-PARSER-PROTOTYPE-2026-10-18.md e docs/evidence/DRIVE-TSV-STREAMING-PENDING-2026-10-19.md.</x:v>
+        <x:v>40% mantido. CSV, TSV, JSON, XLS e XLSX têm validação estrutural em fluxo no pipeline das três fontes aprovadas; CSV também aplica limite de colunas com vírgula e ponto e vírgula. Resumos de estado e contagens por execução são persistidos sem nomes ou conteúdo. A estrutura não interpreta campos das pastas de perdas e frete: todo arquivo fica pendente e nenhum valor alimenta a DRE até existirem contratos aprovados. CSV de Recebimentos Futuros continua sendo o único contrato importado. Faltam identidade técnica, contratos das fontes restantes, interpretação e homologação real. Nenhum arquivo real foi lido ou importado nesta etapa, nenhuma tela nem regra financeira foi alterada. Evidências: docs/evidence/DRIVE-ALL-SOURCE-STRUCTURAL-STREAMING-2026-10-19.md, docs/evidence/DRIVE-XLS-STREAMING-PENDING-2026-10-19.md, docs/evidence/DRIVE-XLSX-XML-TOKEN-LIMIT-2026-10-19.md e docs/evidence/DRIVE-TSV-STREAMING-PENDING-2026-10-19.md.</x:v>
       </x:c>
       <x:c r="I49" s="11" t="str">
         <x:v>Engenharia</x:v>
@@ -6762,7 +6762,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd9b439e3625447ec"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R768857032760479d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9973,7 +9973,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b5ad6b2dc6c4cfb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R230f7fd06b814af1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10398,7 +10398,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc90b8197d3cf4b9b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0cea9dbe6b014c5e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>